<commit_message>
administracion de suscripciones en backoffice
</commit_message>
<xml_diff>
--- a/src/assets/plantilla-catalogo.xlsx
+++ b/src/assets/plantilla-catalogo.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\facub\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\facub\OneDrive\Documents\DesarrolloWeb\ProyectoCatalogo\Varios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7DDBAAA-9CB6-4ADA-AD94-D95C61FE9E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A995CD6A-7B54-4CFD-8586-3B1F8D18793E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B18C3C7B-2DB4-4E4C-A8AC-F28B3A563A95}"/>
   </bookViews>
@@ -63,7 +63,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;\ #,##0"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -88,7 +92,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -96,15 +100,69 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -439,35 +497,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71FF6826-DFDC-4912-A178-FC33BAF5F241}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.625" customWidth="1"/>
-    <col min="2" max="2" width="12.5" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="19.875" customWidth="1"/>
-    <col min="6" max="6" width="19.75" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="41.85546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21" style="2" customWidth="1"/>
+    <col min="4" max="4" width="23.42578125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="20.42578125" style="6" customWidth="1"/>
+    <col min="6" max="6" width="23.5703125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E2" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>